<commit_message>
Update Multiple Locations sheet with Putaway Rule Location column
Added "Putaway Rule Location" column to Sheet 3 showing the assigned
putaway sublocation, or "No Putaway Rule" if none is defined.

https://claude.ai/code/session_01MwzRjCEhdHQynxN2s2xnhJ
</commit_message>
<xml_diff>
--- a/location_analysis.xlsx
+++ b/location_analysis.xlsx
@@ -430,7 +430,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Actual Location</t>
+          <t>Current Location</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -1929,7 +1929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B86"/>
+  <dimension ref="A1:B112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1940,115 +1940,115 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Location(s)</t>
+          <t>Current Location</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>[100009377] OB TARAMA 10 KG</t>
+          <t>[ELBELLOTA] JAMON Iberico Belota Leg Rwpkg</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Main/Stock/C/22/01</t>
+          <t>Main/Stock/D/24/03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>[100344] FB Tasmanian Smoked Salmon Premium Grade 100G</t>
+          <t>[SERRANOBRICK] JAMON Serrano Reserva Brick Rw Pkg</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Main/Stock/Transfer</t>
+          <t>Main/Stock/D/27/01</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>[1009133] LB Traditional Leg Ham 100G</t>
+          <t>[MH144] MH Organic Crispbread With Tomato, Cheese &amp; Sesame 200G</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Main/Stock/A/36/01/A</t>
+          <t>Main/Stock/M/03/01</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>[1009157] LB Mild Sopressa 100G</t>
+          <t>[1808493] FIFYA Pb Hommus 180G</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Main/Stock/A/36/03/A</t>
+          <t>Main/Stock/D/01/02/B</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>[1009164] LB Hot Sopressa 100G</t>
+          <t>[100009377] OB TARAMA 10 KG</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Main/Stock/A/35/03/A</t>
+          <t>Main/Stock/C/22/01</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>[1200701] CB Persian Fetta 1.2Kg</t>
+          <t>[4500814] FIFYA Falafel Balls 4Kg Bucket</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Main/Stock/H/08/01</t>
+          <t>Main/Stock/C/22/01</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>[125357] The Wild Australian Lemon-Myrtle &amp; Sea Salt Rub 125G</t>
+          <t>[4500821] FIFYA Falafel Sesame 4Kg Bucket</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Main/Stock/J/14/02/C</t>
+          <t>Main/Stock/C/22/01</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>[125364] The Wild Argentinian Chimichurri Rub 125G</t>
+          <t>[2500220] IOS Tofu Marinated In Teriyaki Sauce 250G</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Main/Stock/J/14/02/A</t>
+          <t>Main/Stock/A/31/01/B</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>[1808493] FIFYA Pb Hommus 180G</t>
+          <t>[MH124] MH Organic Crispbread With Rustic 3 Seeds 200G</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Main/Stock/D/01/02/B, Main/Stock/D/20/02/C</t>
+          <t>Main/Stock/M/06/01</t>
         </is>
       </c>
     </row>
@@ -2067,12 +2067,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>[2006253] PPC MARINATED GREEN OLIVES 200G</t>
+          <t>[6XMCC0886] MCC Fetta Persian 250Gx6</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Main/Stock/F/04/01/A</t>
+          <t>Main/Stock/Transfer</t>
         </is>
       </c>
     </row>
@@ -2091,84 +2091,84 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>[225081] FIFYA Pb Gf Falafel 250 G</t>
+          <t>[2006253] PPC MARINATED GREEN OLIVES 200G</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Main/Stock/D/06/02/B</t>
+          <t>Main/Stock/F/04/01/A</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>[225814] FIFYA Traditional Falafel Pb 250G</t>
+          <t>[759041] LB Flat Pancetta 75G</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Main/Stock/D/20/02/C</t>
+          <t>Main/Stock/A/35/03/B</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>[225821] FIFYA Falafel With Sesame Pb 250G</t>
+          <t>[1009164] LB Hot Sopressa 100G</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Main/Stock/D/20/02/C, Main/Stock/Transfer</t>
+          <t>Main/Stock/A/35/03/A</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>[2500220] IOS Tofu Marinated In Teriyaki Sauce 250G</t>
+          <t>[1009157] LB Mild Sopressa 100G</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Main/Stock/A/31/01/B</t>
+          <t>Main/Stock/A/36/03/A</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>[2500237] IOS Tofu Marinated In Bbq Sauce 250G</t>
+          <t>[1009133] LB Traditional Leg Ham 100G</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Main/Stock/A/31/02/A</t>
+          <t>Main/Stock/A/36/01/A</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>[2503870] MCC Premium Mascarpone 250G</t>
+          <t>[LE5942] Leon Hot Italian Salami 100G</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/D/20/02/C, Main/Stock/F/14/02, Main/Stock/N/06/01, Main/Stock/Transfer</t>
+          <t>Main/Stock/A/34/01/D</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>[2504218C] FIFYA 3-Layers Nachos Dip 250G (12-Case)</t>
+          <t>[MCC5536X6] MCC Mcc Fetta Dukkah Balls 250Gx6</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/N/06/01, Main/Stock/Transfer</t>
+          <t>Main/Stock/F/11/01</t>
         </is>
       </c>
     </row>
@@ -2187,127 +2187,127 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>[4500814] FIFYA Falafel Balls 4Kg Bucket</t>
+          <t>[2500237] IOS Tofu Marinated In Bbq Sauce 250G</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Main/Stock/C/22/01, Main/Stock/F/14/02, Main/Stock/N/06/01, Main/Stock/Transfer</t>
+          <t>Main/Stock/A/31/02/A</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>[4500821] FIFYA Falafel Sesame 4Kg Bucket</t>
+          <t>[100344] FB Tasmanian Smoked Salmon Premium Grade 100G</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Main/Stock/C/22/01</t>
+          <t>Main/Stock/Transfer</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>[5000754] CB Fetta W Garlic &amp; Herbs 5Kg</t>
+          <t>[125357] The Wild Australian Lemon-Myrtle &amp; Sea Salt Rub 125G</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Main/Stock/D/20/02/C</t>
+          <t>Main/Stock/J/14/02/C</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>[5000DANFET] CB Danish Fetta In Brine 5Kg Bucket</t>
+          <t>[125364] The Wild Argentinian Chimichurri Rub 125G</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Main/Stock/H/08/01</t>
+          <t>Main/Stock/J/14/02/A</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>[6XMCC0886] MCC Fetta Persian 250Gx6</t>
+          <t>[2503870] MCC Premium Mascarpone 250G</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Main/Stock/Transfer</t>
+          <t>Main/Stock/F/14/02</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>[759041] LB Flat Pancetta 75G</t>
+          <t>[BLUESTRAPPING] BLUE MACHINE STRAPPING 120MM*3000MM</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Main/Stock/A/35/03/B</t>
+          <t>Main/Stock/F/14/02</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>[ANCHOVIES WHITE] ANCHOVIES WHITE</t>
+          <t>[MCC2651] MCC Labneh With Zataar &amp; Sumac 250G</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Main/Stock/F/14/02</t>
+          <t>Main/Stock/D/20/02/C</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>[AUSFET13KG] CB Australian Fetta  Bucket</t>
+          <t>[1808493] FIFYA Pb Hommus 180G</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Main/Stock/F/14/02</t>
+          <t>Main/Stock/D/20/02/C</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>[AUSPARMB] CB AUSTRALIAN PARMESAN R/W WHEEL</t>
+          <t>[AUSFET13KG] CB Australian Fetta  Bucket</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Main/Stock/F/14/02, Main/Stock/H/07/01</t>
+          <t>Main/Stock/F/14/02</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>[BLUESTRAPPING] BLUE MACHINE STRAPPING 120MM*3000MM</t>
+          <t>[225821] FIFYA Falafel With Sesame Pb 250G</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Main/Stock/F/14/02</t>
+          <t>Main/Stock/D/20/02/C</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>[BULGARIAN FETTA] BULGARIAN FETTA</t>
+          <t>[PURCHARN] CB Charnwod Smoked Cheese 1/2 Wheel Pkg</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2319,79 +2319,79 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>[CBSTYOG10] CB: AUTHENTIC STRAINED YOGHURT 10 KG</t>
+          <t>[AUSPARMB] CB AUSTRALIAN PARMESAN R/W WHEEL</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Main/Stock</t>
+          <t>Main/Stock/F/14/02</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>[DUKKA] OB Dukka Traditional 1Kg</t>
+          <t>[PURGOUDA] CB Gouda Cheese Full Whel Pkg</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Main/Stock/N/06/01</t>
+          <t>Main/Stock/F/14/02</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>[DUTCHGOUDA18B] CB Dutch Weydeland Flinck Gouda Aged 18 Months 12Kg</t>
+          <t>[PURSHEEPTRU] SPANISH SHEEP CHESE WITH TRUFFLE PKG</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Main/Stock/H/07/02</t>
+          <t>Main/Stock/F/14/02</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>[ELBELLOTA] JAMON Iberico Belota Leg Rwpkg</t>
+          <t>[4500814] FIFYA Falafel Balls 4Kg Bucket</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Main/Stock/D/24/03</t>
+          <t>Main/Stock/F/14/02</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>[FREIGHT] DELIVERY CHARGE</t>
+          <t>[PURDANISHBLUE] CB Danish Blue Cheese Whel Pkg</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/N/06/01</t>
+          <t>Main/Stock/F/14/02</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>[GLOVESFREEZER] GLOVES FREEZER NINJA ICE LRG</t>
+          <t>[GOATSTRUFF] CB Dutch Goats Cheese With Truffle Rw Pcs (Ctn-8)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Main/Stock/D/20/02/C</t>
+          <t>Main/Stock/F/14/02</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>[GOATSTRUFF] CB Dutch Goats Cheese With Truffle Rw Pcs (Ctn-8)</t>
+          <t>[PONIBROPEE10KG] ONION BROWM PEELD DICED</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2403,151 +2403,151 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>[GOUDACUMIN] CB Dutch Spiced Gouda With Cumin Seeds Rw Pcs (Ctn-8)</t>
+          <t>[ANCHOVIES WHITE] ANCHOVIES WHITE</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Main/Stock/D/20/02/C, Main/Stock/N/06/01</t>
+          <t>Main/Stock/F/14/02</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>[HALOUMIB10KG] CB Australian Halloumi Bulk 10kg</t>
+          <t>[BULGARIAN FETTA] BULGARIAN FETTA</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Main/Stock/H/06/01</t>
+          <t>Main/Stock/F/14/02</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>[LE5942] Leon Hot Italian Salami 100G</t>
+          <t>[5000754] CB Fetta W Garlic &amp; Herbs 5Kg</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Main/Stock/A/34/01/D</t>
+          <t>Main/Stock/D/20/02/C</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>[MCC2651] MCC Labneh With Zataar &amp; Sumac 250G</t>
+          <t>[MCC5536] MCC Fetta Dukkah Balls 250G</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Main/Stock/D/20/02/C, Main/Stock/N/06/01</t>
+          <t>Main/Stock/D/20/02/C</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>[MCC5536X6] MCC Mcc Fetta Dukkah Balls 250Gx6</t>
+          <t>[2503870] MCC Premium Mascarpone 250G</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Main/Stock/F/11/01</t>
+          <t>Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>[MCC5536] MCC Fetta Dukkah Balls 250G</t>
+          <t>[PURGORGON] CB GORGONZOLA DOLCEE FULL PKG</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Main/Stock/D/20/02/C</t>
+          <t>Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>[MH124] MH Organic Crispbread With Rustic 3 Seeds 200G</t>
+          <t>[PUREDAMDUTCH] CB Dutch Edam Cheese Red Bal Pkg</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Main/Stock/M/06/01</t>
+          <t>Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>[MH144] MH Organic Crispbread With Tomato, Cheese &amp; Sesame 200G</t>
+          <t>[PURMASDAAM] CB MASDAM CHEESE FULL WHEL RW PKG</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Main/Stock/M/03/01</t>
+          <t>Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>[ORGTRUFFLEB] CB: Aged Organic Dutch Truffle Cheese Bulk</t>
+          <t>[PURASIAGO] CB ASIAGO CHEESE FULL WHEL RW PKG</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Main/Stock/H/07/02</t>
+          <t>Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>[PONIBROPEE10KG] ONION BROWM PEELD DICED</t>
+          <t>[PURDANISHBLUE] CB Danish Blue Cheese Whel Pkg</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Main/Stock/F/14/02</t>
+          <t>Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>[PROVDOLB] CB PROVOLONE DOLCE FULL RW</t>
+          <t>[DUKKA] OB Dukka Traditional 1Kg</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Main/Stock/H/06/01</t>
+          <t>Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>[PURAMBROS] CB Ambrosia Cheese Full Whel Pkg</t>
+          <t>[GOUDACUMIN] CB Dutch Spiced Gouda With Cumin Seeds Rw Pcs (Ctn-8)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Main/Stock/H/06/02</t>
+          <t>Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>[PURASIAGO] CB ASIAGO CHEESE FULL WHEL RW PKG</t>
+          <t>[FREIGHT] DELIVERY CHARGE</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2559,223 +2559,223 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>[PURAUSPARM] CB AUSTRALIAN PARMESAN R/W WHEL</t>
+          <t>[4500814] FIFYA Falafel Balls 4Kg Bucket</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Main/Stock/H/07/01</t>
+          <t>Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>[PURAUSPECCH] CB Australian Pecorino Chilli Whel Pkg</t>
+          <t>[2504218C] FIFYA 3-Layers Nachos Dip 250G (12-Case)</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Main/Stock</t>
+          <t>Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>[PURAUSPECPEP] CB AUSTRALIAN PECORINO PEPPER WHEL PKG</t>
+          <t>[MCC2651] MCC Labneh With Zataar &amp; Sumac 250G</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/H/06/02</t>
+          <t>Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>[PURAUSPEC] CB AUSTRALIAN PECORINO WHEL PKG</t>
+          <t>[GOUDACUMIN] CB Dutch Spiced Gouda With Cumin Seeds Rw Pcs (Ctn-8)</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/H/06/02</t>
+          <t>Main/Stock/D/20/02/C</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>[PURBOBBK] BOB Black Knight Extra Mature Cheddar Loaf 1.2 To 1.5 Kg R/W</t>
+          <t>[225814] FIFYA Traditional Falafel Pb 250G</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Main/Stock/H/06/02</t>
+          <t>Main/Stock/D/20/02/C</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>[PURBOBRR] BOB Red Ribbon Vintage Red Leicster Loaf 1.2 To 1.5 Kg R/W</t>
+          <t>[2503870] MCC Premium Mascarpone 250G</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Main/Stock/H/06/02</t>
+          <t>Main/Stock/D/20/02/C</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>[PURCHARN] CB Charnwod Smoked Cheese 1/2 Wheel Pkg</t>
+          <t>[2503870] MCC Premium Mascarpone 250G</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/F/14/02</t>
+          <t>Main/Stock/Transfer</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>[PURCHEDDARB] CB Cheddar Chees Bulk Pkg</t>
+          <t>[225821] FIFYA Falafel With Sesame Pb 250G</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Main/Stock/H/06/02</t>
+          <t>Main/Stock/Transfer</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>[PURDANISHBLUE] CB Danish Blue Cheese Whel Pkg</t>
+          <t>[4500814] FIFYA Falafel Balls 4Kg Bucket</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Main/Stock/F/14/02, Main/Stock/H/06/02, Main/Stock/N/06/01</t>
+          <t>Main/Stock/Transfer</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>[PURDUTCHGOUDA] CB Dutch Weydland Flinck Gouda Aged 18 Months 12Kg</t>
+          <t>[2504218C] FIFYA 3-Layers Nachos Dip 250G (12-Case)</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Main/Stock/H/07/01</t>
+          <t>Main/Stock/Transfer</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>[PUREDAMDUTCH] CB Dutch Edam Cheese Red Bal Pkg</t>
+          <t>[2504218C] FIFYA 3-Layers Nachos Dip 250G (12-Case)</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Main/Stock/H/06/02, Main/Stock/N/06/01</t>
+          <t>Main/Stock</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>[PUREMMENTAL] CB Emmental Chese Full Piece Pkg</t>
+          <t>[GLOVESFREEZER] GLOVES FREEZER NINJA ICE LRG</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Main/Stock/H/06/02</t>
+          <t>Main/Stock/D/20/02/C</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>[PURESROM] CB ESROM DANISH CHEESE FULL WHEL PKG</t>
+          <t>[2503870] MCC Premium Mascarpone 250G</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/H/06/02</t>
+          <t>Main/Stock</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>[PURFONTINA] CB Danish Fontina Cheese  Wheel Rw Pkg</t>
+          <t>[1200701] CB Persian Fetta 1.2Kg</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Main/Stock/H/06/02</t>
+          <t>Main/Stock/H/08/01</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>[PURFRICO] CB Dutch Frico Smoked Cheese Whel Pkg</t>
+          <t>[5000DANFET] CB Danish Fetta In Brine 5Kg Bucket</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Main/Stock/H/06/02</t>
+          <t>Main/Stock/H/08/01</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>[PURGORGON] CB GORGONZOLA DOLCEE FULL PKG</t>
+          <t>[PROVDOLB] CB PROVOLONE DOLCE FULL RW</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Main/Stock/N/06/01</t>
+          <t>Main/Stock/H/06/01</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>[PURGORGPIC] CB GORGONZOLA PICCANTE WHEL PKG</t>
+          <t>[HALOUMIB10KG] CB Australian Halloumi Bulk 10kg</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Main/Stock</t>
+          <t>Main/Stock/H/06/01</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>[PURGOUDA] CB Gouda Cheese Full Whel Pkg</t>
+          <t>[PURBOBBK] BOB Black Knight Extra Mature Cheddar Loaf 1.2 To 1.5 Kg R/W</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Main/Stock/F/14/02, Main/Stock/H/06/02</t>
+          <t>Main/Stock/H/06/02</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>[PURGRANA] CB Grana Padano Full Whel Rw Pkg</t>
+          <t>[PURBOBRR] BOB Red Ribbon Vintage Red Leicster Loaf 1.2 To 1.5 Kg R/W</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2787,7 +2787,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>[PURGRUYERE] CB Swiss Gruyere Chese Full Piece Rw Pkg</t>
+          <t>[PURDANISHBLUE] CB Danish Blue Cheese Whel Pkg</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2799,7 +2799,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>[PURHAVARTI] CB Havarti Cheese Full Piece Rw PkG</t>
+          <t>[PURVINTAGEB] ENGLISH Vintage Chedar Wheel Pkg</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2811,7 +2811,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>[PURKEFALO] CB Kefalo Greviera Full Whel Rw Pkg</t>
+          <t>[PURMANCHEGO3] CB Manchego 3 Month Bulk Pkg</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2823,19 +2823,19 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>[PURMANCHEGO12] CB MANCHEGO AGED 12 MONTHS WHEL PKG</t>
+          <t>[PURWALNUT] CB Walnut Chese Wheel Pkg</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/H/06/02</t>
+          <t>Main/Stock/H/06/02</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>[PURMANCHEGO3] CB Manchego 3 Month Bulk Pkg</t>
+          <t>[PURSPGOAT] CB Spanish Goat Chese Semihard Wheel Pkg</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2847,19 +2847,19 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>[PURMASDAAM] CB MASDAM CHEESE FULL WHEL RW PKG</t>
+          <t>[PURGOUDA] CB Gouda Cheese Full Whel Pkg</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Main/Stock/N/06/01</t>
+          <t>Main/Stock/H/06/02</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>[PURMOZZAR] CB Australian Caterers Mozzarela Bulk Pk</t>
+          <t>[PUREMMENTAL] CB Emmental Chese Full Piece Pkg</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2871,7 +2871,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>[PURPECOROM] CB Pecorino Romano Full Whel</t>
+          <t>[PURREGGIAN] CB REGGIANO PARMEGIANO FULL WHEL RW PKG</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2883,7 +2883,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>[PURREGGIAN] CB REGGIANO PARMEGIANO FULL WHEL RW PKG</t>
+          <t>[PURHAVARTI] CB Havarti Cheese Full Piece Rw PkG</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2895,19 +2895,19 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>[PURSHEEPTRU] SPANISH SHEEP CHESE WITH TRUFFLE PKG</t>
+          <t>[PURGRANA] CB Grana Padano Full Whel Rw Pkg</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Main/Stock/F/14/02</t>
+          <t>Main/Stock/H/06/02</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>[PURSPGOAT] CB Spanish Goat Chese Semihard Wheel Pkg</t>
+          <t>[PURCHEDDARB] CB Cheddar Chees Bulk Pkg</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2919,48 +2919,360 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>[PURTASTY] CB Tasty Chese Bulk Pkg</t>
+          <t>[PURFRICO] CB Dutch Frico Smoked Cheese Whel Pkg</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Main/Stock</t>
+          <t>Main/Stock/H/06/02</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>[PURVINTAGEB] ENGLISH Vintage Chedar Wheel Pkg</t>
+          <t>[PURAUSPECPEP] CB AUSTRALIAN PECORINO PEPPER WHEL PKG</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/H/06/02</t>
+          <t>Main/Stock/H/06/02</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>[PURWALNUT] CB Walnut Chese Wheel Pkg</t>
+          <t>[PURAUSPEC] CB AUSTRALIAN PECORINO WHEL PKG</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/H/06/02</t>
+          <t>Main/Stock/H/06/02</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>[SERRANOBRICK] JAMON Serrano Reserva Brick Rw Pkg</t>
+          <t>[PURPECOROM] CB Pecorino Romano Full Whel</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Main/Stock/D/27/01</t>
+          <t>Main/Stock/H/06/02</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>[PURMANCHEGO12] CB MANCHEGO AGED 12 MONTHS WHEL PKG</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Main/Stock/H/06/02</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>[PURAMBROS] CB Ambrosia Cheese Full Whel Pkg</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Main/Stock/H/06/02</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>[PURFONTINA] CB Danish Fontina Cheese  Wheel Rw Pkg</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Main/Stock/H/06/02</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>[PURESROM] CB ESROM DANISH CHEESE FULL WHEL PKG</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Main/Stock/H/06/02</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>[PURGRUYERE] CB Swiss Gruyere Chese Full Piece Rw Pkg</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Main/Stock/H/06/02</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>[PURMOZZAR] CB Australian Caterers Mozzarela Bulk Pk</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Main/Stock/H/06/02</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>[PUREDAMDUTCH] CB Dutch Edam Cheese Red Bal Pkg</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Main/Stock/H/06/02</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>[PURKEFALO] CB Kefalo Greviera Full Whel Rw Pkg</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Main/Stock/H/06/02</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>[AUSPARMB] CB AUSTRALIAN PARMESAN R/W WHEEL</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Main/Stock/H/07/01</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>[PURDUTCHGOUDA] CB Dutch Weydland Flinck Gouda Aged 18 Months 12Kg</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Main/Stock/H/07/01</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>[PURAUSPARM] CB AUSTRALIAN PARMESAN R/W WHEL</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Main/Stock/H/07/01</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>[DUTCHGOUDA18B] CB Dutch Weydeland Flinck Gouda Aged 18 Months 12Kg</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Main/Stock/H/07/02</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>[ORGTRUFFLEB] CB: Aged Organic Dutch Truffle Cheese Bulk</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Main/Stock/H/07/02</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>[CBSTYOG10] CB: AUTHENTIC STRAINED YOGHURT 10 KG</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Main/Stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>[225081] FIFYA Pb Gf Falafel 250 G</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Main/Stock/D/06/02/B</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>[PURAUSPEC] CB AUSTRALIAN PECORINO WHEL PKG</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Main/Stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>[PURAUSPECCH] CB Australian Pecorino Chilli Whel Pkg</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Main/Stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>[PURAUSPECPEP] CB AUSTRALIAN PECORINO PEPPER WHEL PKG</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Main/Stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>[PURTASTY] CB Tasty Chese Bulk Pkg</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Main/Stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>[FREIGHT] DELIVERY CHARGE</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Main/Stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>[PURESROM] CB ESROM DANISH CHEESE FULL WHEL PKG</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Main/Stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>[PURCHARN] CB Charnwod Smoked Cheese 1/2 Wheel Pkg</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Main/Stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>[PURGORGPIC] CB GORGONZOLA PICCANTE WHEL PKG</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Main/Stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>[PURMANCHEGO12] CB MANCHEGO AGED 12 MONTHS WHEL PKG</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Main/Stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>[PURVINTAGEB] ENGLISH Vintage Chedar Wheel Pkg</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Main/Stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>[PURWALNUT] CB Walnut Chese Wheel Pkg</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Main/Stock</t>
         </is>
       </c>
     </row>
@@ -2975,7 +3287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:D69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2991,6 +3303,11 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Putaway Rule Location</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>All Locations</t>
         </is>
       </c>
@@ -3006,6 +3323,11 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Main/Stock/J/09/02</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>Main/Stock, Main/Stock/J/09/02</t>
         </is>
       </c>
@@ -3021,6 +3343,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Main/Stock/H/02/02/B</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>Main/Stock/H/02/02/B, Main/Stock/H/08/02</t>
         </is>
       </c>
@@ -3028,7 +3355,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>[1750329] LB Cured Tasty Chorizo 175G</t>
+          <t>[1208240] BOB Oak Smoked Mature Cheddar 120G Wedge</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -3036,14 +3363,19 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Main/Stock/C/02/02, Main/Stock/D/24/01</t>
+          <t>Main/Stock/H/08/02</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Main/Stock/H/02/02/B, Main/Stock/H/08/02</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>[1750336] LB Cured Chilli Chorizo 175G</t>
+          <t>[1750329] LB Cured Tasty Chorizo 175G</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -3051,14 +3383,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Main/Stock/C/01/02, Main/Stock/D/22/01</t>
+          <t>Main/Stock/C/02/02</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Main/Stock/C/02/02, Main/Stock/D/24/01</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>[1808493] FIFYA Pb Hommus 180G</t>
+          <t>[1750336] LB Cured Chilli Chorizo 175G</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -3066,14 +3403,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Main/Stock/D/01/02/B, Main/Stock/D/20/02/C</t>
+          <t>Main/Stock/C/01/02</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Main/Stock/C/01/02, Main/Stock/D/22/01</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>[200033] OB Crunchy Romesco  200G</t>
+          <t>[1808493] FIFYA Pb Hommus 180G</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -3081,14 +3423,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Main/Stock/A/19/02, Main/Stock/A/22/01</t>
+          <t>No Putaway Rule</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Main/Stock/D/01/02/B, Main/Stock/D/20/02/C</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>[2001915] OB Marinated Capsicum &amp; Roasted Eggplant  200G</t>
+          <t>[200033] OB Crunchy Romesco  200G</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -3096,14 +3443,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Main/Stock/A/23/02, Main/Stock/A/24/02</t>
+          <t>Main/Stock/A/19/02</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Main/Stock/A/19/02, Main/Stock/A/22/01</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>[2008861] OB Crunchy Basil  200G</t>
+          <t>[2001915] OB Marinated Capsicum &amp; Roasted Eggplant  200G</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -3111,14 +3463,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Main/Stock/A/08/01, Main/Stock/A/12/02</t>
+          <t>Main/Stock/A/24/02</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Main/Stock/A/23/02, Main/Stock/A/24/02</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>[2008946] OB Beetroot Indulgence  200G</t>
+          <t>[2008861] OB Crunchy Basil  200G</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -3126,14 +3483,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Main/Stock/A/04/01, Main/Stock/A/14/02</t>
+          <t>Main/Stock/A/12/02</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Main/Stock/A/08/01, Main/Stock/A/12/02</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>[2009011] OB Crunchy Spicy Pumpkin  200G</t>
+          <t>[2008946] OB Beetroot Indulgence  200G</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -3141,74 +3503,99 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Main/Stock/A/08/01, Main/Stock/A/11/01</t>
+          <t>Main/Stock/A/14/02</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Main/Stock/A/04/01, Main/Stock/A/14/02</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>[22001212] OB Dip Sweet Chilli Crab Dip 2.2Kg</t>
+          <t>[2009011] OB Crunchy Spicy Pumpkin  200G</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Main/Stock/D/20/02/C, Main/Stock/E/13/01, Main/Stock/F/14/02</t>
+          <t>Main/Stock/A/08/01</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Main/Stock/A/08/01, Main/Stock/A/11/01</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>[2200149] FIFYA Crunchy Moroccan Harissa 2.2K</t>
+          <t>[22001212] OB Dip Sweet Chilli Crab Dip 2.2Kg</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Main/Stock/E/14/01, Main/Stock/N/06/01</t>
+          <t>Main/Stock/E/13/01</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Main/Stock/D/20/02/C, Main/Stock/E/13/01, Main/Stock/F/14/02</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>[22001] FIFYA Middle Eastern Hommus 2.2Kg</t>
+          <t>[2200149] FIFYA Crunchy Moroccan Harissa 2.2K</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Main/Stock/D/20/02/C, Main/Stock/E/15/01, Main/Stock/N/06/01</t>
+          <t>Main/Stock/E/14/01</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Main/Stock/E/14/01, Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>[22002417] CB Persian Fetta 2.2Kg</t>
+          <t>[22001] FIFYA Middle Eastern Hommus 2.2Kg</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Main/Stock/E/10/01, Main/Stock/F/14/02</t>
+          <t>Main/Stock/E/15/01</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Main/Stock/D/20/02/C, Main/Stock/E/15/01, Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>[2200407] FIFYA Mediter Basil Pesto 2.2Kg</t>
+          <t>[22002417] CB Persian Fetta 2.2Kg</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -3216,14 +3603,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Main/Stock/E/15/01, Main/Stock/N/06/01</t>
+          <t>Main/Stock/E/10/01</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Main/Stock/E/10/01, Main/Stock/F/14/02</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>[2200414] OB Sundried Tomato Pesto 2.2Kg</t>
+          <t>[2200407] FIFYA Mediter Basil Pesto 2.2Kg</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -3231,14 +3623,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Main/Stock/D/20/02/C, Main/Stock/E/13/01</t>
+          <t>Main/Stock/E/15/01</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Main/Stock/E/15/01, Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>[2200455] CB Goat Cheese Garlic &amp; Herbs 2.2Kg</t>
+          <t>[2200414] OB Sundried Tomato Pesto 2.2Kg</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -3246,14 +3643,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Main/Stock/E/09/01, Main/Stock/N/06/01</t>
+          <t>Main/Stock/E/13/01</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Main/Stock/D/20/02/C, Main/Stock/E/13/01</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>[22005233] FIFYA Vegan Ptato,Crindr,Chili2.2Kg</t>
+          <t>[2200455] CB Goat Cheese Garlic &amp; Herbs 2.2Kg</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -3261,14 +3663,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Main/Stock/E/14/01, Main/Stock/F/14/02</t>
+          <t>Main/Stock/E/09/01</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Main/Stock/E/09/01, Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>[22005240] FIFYA Vegan Pumpkin,Herb&amp;Seeds2.2Kg</t>
+          <t>[22005233] FIFYA Vegan Ptato,Crindr,Chili2.2Kg</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -3276,14 +3683,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Main/Stock/D/20/02/C, Main/Stock/E/15/01</t>
+          <t>Main/Stock/E/14/01</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Main/Stock/E/14/01, Main/Stock/F/14/02</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>[22006774] OB Bruschetta Mix 2.2Kg</t>
+          <t>[22005240] FIFYA Vegan Pumpkin,Herb&amp;Seeds2.2Kg</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -3291,14 +3703,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Main/Stock/E/12/01, Main/Stock/F/14/02</t>
+          <t>Main/Stock/E/15/01</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Main/Stock/D/20/02/C, Main/Stock/E/15/01</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>[2200807] FF Rstd Caps Parmesan &amp; Chives 2.2K</t>
+          <t>[22006774] OB Bruschetta Mix 2.2Kg</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -3306,74 +3723,99 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Main/Stock/E/14/01, Main/Stock/F/14/02</t>
+          <t>Main/Stock/E/12/01</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Main/Stock/E/12/01, Main/Stock/F/14/02</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>[2200838] FIFYA Crunchy Basil 2.2Kg</t>
+          <t>[2200807] FF Rstd Caps Parmesan &amp; Chives 2.2K</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Main/Stock/D/20/02/C, Main/Stock/E/14/01, Main/Stock/N/06/01</t>
+          <t>Main/Stock/E/14/01</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Main/Stock/E/14/01, Main/Stock/F/14/02</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>[22008793] OB Dip Traditional Hommus 2.2Kg</t>
+          <t>[2200838] FIFYA Crunchy Basil 2.2Kg</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Main/Stock/E/13/01, Main/Stock/N/06/01</t>
+          <t>Main/Stock/E/14/01</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Main/Stock/D/20/02/C, Main/Stock/E/14/01, Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>[22009836] OB Dip Gourmet Tarama 2.2Kg</t>
+          <t>[22008793] OB Dip Traditional Hommus 2.2Kg</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Main/Stock/E/12/01, Main/Stock/F/14/02, Main/Stock/N/06/01</t>
+          <t>Main/Stock/E/13/01</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Main/Stock/E/13/01, Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>[225371] FIFYA French Onion Dip  200G</t>
+          <t>[22009836] OB Dip Gourmet Tarama 2.2Kg</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Main/Stock/B/02/01, Main/Stock/B/05/02/A</t>
+          <t>Main/Stock/E/12/01</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Main/Stock/E/12/01, Main/Stock/F/14/02, Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>[225821] FIFYA Falafel With Sesame Pb 250G</t>
+          <t>[225371] FIFYA French Onion Dip  200G</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -3381,44 +3823,59 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Main/Stock/D/20/02/C, Main/Stock/Transfer</t>
+          <t>Main/Stock/B/02/01</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Main/Stock/B/02/01, Main/Stock/B/05/02/A</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>[2501234] FIFYA Pb Beetroot Hommus   250G</t>
+          <t>[225821] FIFYA Falafel With Sesame Pb 250G</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Main/Stock/A/28/01, Main/Stock/B/28/01, Main/Stock/B/29/02</t>
+          <t>No Putaway Rule</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Main/Stock/D/20/02/C, Main/Stock/Transfer</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>[2502059] OB Heavenly Spicy Trio  250G</t>
+          <t>[2501234] FIFYA Pb Beetroot Hommus   250G</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Main/Stock/A/11/01, Main/Stock/A/12/02</t>
+          <t>Main/Stock/B/28/01</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Main/Stock/A/28/01, Main/Stock/B/28/01, Main/Stock/B/29/02</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>[2502408] LB Saucisson Sec Salami 250G</t>
+          <t>[2502059] OB Heavenly Spicy Trio  250G</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -3426,74 +3883,99 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Main/Stock/D/01/01, Main/Stock/D/01/02</t>
+          <t>Main/Stock/A/11/01</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Main/Stock/A/11/01, Main/Stock/A/12/02</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>[2503870] MCC Premium Mascarpone 250G</t>
+          <t>[2502408] LB Saucisson Sec Salami 250G</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/D/20/02/C, Main/Stock/F/14/02, Main/Stock/N/06/01, Main/Stock/Transfer</t>
+          <t>Main/Stock/D/01/02</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Main/Stock/D/01/01, Main/Stock/D/01/02</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>[250396] OB Traditional Semi Sundried Tomatoes 335G</t>
+          <t>[2503870] MCC Premium Mascarpone 250G</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Main/Stock/D/17/01, Main/Stock/F/01/01/A</t>
+          <t>No Putaway Rule</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Main/Stock, Main/Stock/D/20/02/C, Main/Stock/F/14/02, Main/Stock/N/06/01, Main/Stock/Transfer</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>[2504218C] FIFYA 3-Layers Nachos Dip 250G (12-Case)</t>
+          <t>[250396] OB Traditional Semi Sundried Tomatoes 335G</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/N/06/01, Main/Stock/Transfer</t>
+          <t>Main/Stock/D/17/01</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Main/Stock/D/17/01, Main/Stock/F/01/01/A</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>[2505240] FIFYA Pb Roasted Pumpkin With Fresh Herbs And Seeds 250G</t>
+          <t>[2504218C] FIFYA 3-Layers Nachos Dip 250G (12-Case)</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Main/Stock/B/20/01, Main/Stock/E/22/01/C</t>
+          <t>No Putaway Rule</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Main/Stock, Main/Stock/N/06/01, Main/Stock/Transfer</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>[2505257] FIFYA Pb Basil, Spinach &amp; Roasted Cashew Pesto 250G</t>
+          <t>[2505240] FIFYA Pb Roasted Pumpkin With Fresh Herbs And Seeds 250G</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -3501,14 +3983,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Main/Stock/B/19/01, Main/Stock/B/23/01</t>
+          <t>Main/Stock/B/20/01</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Main/Stock/B/20/01, Main/Stock/E/22/01/C</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>[2506552] CB Persian Fetta With Chilli &amp; Saffron 335G</t>
+          <t>[2505257] FIFYA Pb Basil, Spinach &amp; Roasted Cashew Pesto 250G</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -3516,14 +4003,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/C/06/01</t>
+          <t>Main/Stock/B/19/01</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Main/Stock/B/19/01, Main/Stock/B/23/01</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>[2507406] OB Pitted Kalamata Olives With Fresh Lemon, Garlic &amp; Herbs</t>
+          <t>[2506552] CB Persian Fetta With Chilli &amp; Saffron 335G</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -3531,14 +4023,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Main/Stock/F/02/02/B, Main/Stock/H/10/01</t>
+          <t>Main/Stock/C/06/01</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Main/Stock, Main/Stock/C/06/01</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>[250761] CB Fetta Dukkah Balls 335G</t>
+          <t>[2507406] OB Pitted Kalamata Olives With Fresh Lemon, Garlic &amp; Herbs</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -3546,14 +4043,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/C/08/01</t>
+          <t>Main/Stock/D/10/01</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Main/Stock/F/02/02/B, Main/Stock/H/10/01</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>[2507987] OB Dolmades  335G</t>
+          <t>[250761] CB Fetta Dukkah Balls 335G</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -3561,14 +4063,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Main/Stock/D/18/01/A, Main/Stock/F/02/02/A</t>
+          <t>Main/Stock/C/08/01</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Main/Stock, Main/Stock/C/08/01</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>[2509904] OB Gourmet Garlic Dip Skordalia 250G</t>
+          <t>[2507987] OB Dolmades  335G</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -3576,14 +4083,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Main/Stock/A/19/02, Main/Stock/A/22/01</t>
+          <t>Main/Stock/D/18/01/A</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Main/Stock/D/18/01/A, Main/Stock/F/02/02/A</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>[2803733] MCC Persian Goat Cheese 280G</t>
+          <t>[2509904] OB Gourmet Garlic Dip Skordalia 250G</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -3591,44 +4103,59 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Main/Stock/F/12/01, Main/Stock/F/14/02/B</t>
+          <t>Main/Stock/A/22/01</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Main/Stock/A/19/02, Main/Stock/A/22/01</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>[4500814] FIFYA Falafel Balls 4Kg Bucket</t>
+          <t>[2803733] MCC Persian Goat Cheese 280G</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Main/Stock/C/22/01, Main/Stock/F/14/02, Main/Stock/N/06/01, Main/Stock/Transfer</t>
+          <t>Main/Stock/F/14/02/B</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Main/Stock/F/12/01, Main/Stock/F/14/02/B</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>[5506130] OB Heavenly Crunchy Trio Dip Party Size 550G</t>
+          <t>[4500814] FIFYA Falafel Balls 4Kg Bucket</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/E/21/02</t>
+          <t>No Putaway Rule</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Main/Stock/C/22/01, Main/Stock/F/14/02, Main/Stock/N/06/01, Main/Stock/Transfer</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>[AMBROSIA] CB Ambrosia Cheese Rw Pcs (Ctn-8)</t>
+          <t>[5506130] OB Heavenly Crunchy Trio Dip Party Size 550G</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -3636,14 +4163,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Main/Stock/D/20/02/C, Main/Stock/H/14/01/D</t>
+          <t>Main/Stock/E/21/02</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Main/Stock, Main/Stock/E/21/02</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>[AUSPARMB] CB AUSTRALIAN PARMESAN R/W WHEEL</t>
+          <t>[AMBROSIA] CB Ambrosia Cheese Rw Pcs (Ctn-8)</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -3651,14 +4183,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Main/Stock/F/14/02, Main/Stock/H/07/01</t>
+          <t>Main/Stock/H/14/01/D</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Main/Stock/D/20/02/C, Main/Stock/H/14/01/D</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>[BOBBKXMCHRWL] BOB Black Knight Extra Mature Cheddar Loaf 1.2 To 1.5 Kg R/W</t>
+          <t>[AUSPARMB] CB AUSTRALIAN PARMESAN R/W WHEEL</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -3666,20 +4203,30 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/H/07/01</t>
+          <t>No Putaway Rule</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Main/Stock/F/14/02, Main/Stock/H/07/01</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>[BOBRRVRLRWL] BOB Red Ribbon Vintage Red Leicester Loaf 1.2 To 1.5 Kg R/W</t>
+          <t>[BOBBKXMCHRWL] BOB Black Knight Extra Mature Cheddar Loaf 1.2 To 1.5 Kg R/W</t>
         </is>
       </c>
       <c r="B47" t="n">
         <v>2</v>
       </c>
       <c r="C47" t="inlineStr">
+        <is>
+          <t>Main/Stock/H/07/01</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
         <is>
           <t>Main/Stock, Main/Stock/H/07/01</t>
         </is>
@@ -3688,37 +4235,47 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>[EMMENTALB] CB Emmental Cheese Full Piece Pkg</t>
+          <t>[BOBRRVRLRWL] BOB Red Ribbon Vintage Red Leicester Loaf 1.2 To 1.5 Kg R/W</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Main/Stock/D/20/02/C, Main/Stock/F/14/02, Main/Stock/H/07/02, Main/Stock/N/06/01</t>
+          <t>Main/Stock/H/07/01</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Main/Stock, Main/Stock/H/07/01</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>[FREIGHT] DELIVERY CHARGE</t>
+          <t>[EMMENTALB] CB Emmental Cheese Full Piece Pkg</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/N/06/01</t>
+          <t>Main/Stock/H/07/02</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Main/Stock/D/20/02/C, Main/Stock/F/14/02, Main/Stock/H/07/02, Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>[GOUDACUMIN] CB Dutch Spiced Gouda With Cumin Seeds Rw Pcs (Ctn-8)</t>
+          <t>[FREIGHT] DELIVERY CHARGE</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -3726,14 +4283,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Main/Stock/D/20/02/C, Main/Stock/N/06/01</t>
+          <t>No Putaway Rule</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Main/Stock, Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>[GRANA] CB Grana Padano Italian Parmesan Rw Pcs (Ctn-8)</t>
+          <t>[GOUDACUMIN] CB Dutch Spiced Gouda With Cumin Seeds Rw Pcs (Ctn-8)</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -3741,14 +4303,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Main/Stock/H/11/01/D, Main/Stock/Transfer</t>
+          <t>No Putaway Rule</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Main/Stock/D/20/02/C, Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>[HAVARTIB] CB Havarti Cheese Full Piece Rw Pk</t>
+          <t>[GRANA] CB Grana Padano Italian Parmesan Rw Pcs (Ctn-8)</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -3756,14 +4323,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/H/06/01</t>
+          <t>Main/Stock/H/11/01/D</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Main/Stock/H/11/01/D, Main/Stock/Transfer</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>[HAVARTI] CB Havarti Cheese Rw Pcs (Ctn-8)</t>
+          <t>[HAVARTIB] CB Havarti Cheese Full Piece Rw Pk</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -3771,14 +4343,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Main/Stock/H/06/01, Main/Stock/H/10/01/A</t>
+          <t>Main/Stock/H/06/01</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Main/Stock, Main/Stock/H/06/01</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>[MCC2651] MCC Labneh With Zataar &amp; Sumac 250G</t>
+          <t>[HAVARTI] CB Havarti Cheese Rw Pcs (Ctn-8)</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -3786,14 +4363,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Main/Stock/D/20/02/C, Main/Stock/N/06/01</t>
+          <t>Main/Stock/H/10/01/A</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Main/Stock/H/06/01, Main/Stock/H/10/01/A</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>[PURAUSPECPEP] CB AUSTRALIAN PECORINO PEPPER WHEL PKG</t>
+          <t>[HAVARTI] CB Havarti Cheese Rw Pcs (Ctn-8)</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -3801,14 +4383,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/H/06/02</t>
+          <t>Main/Stock/H/06/01</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Main/Stock/H/06/01, Main/Stock/H/10/01/A</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>[PURAUSPEC] CB AUSTRALIAN PECORINO WHEL PKG</t>
+          <t>[MCC2651] MCC Labneh With Zataar &amp; Sumac 250G</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -3816,14 +4403,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/H/06/02</t>
+          <t>No Putaway Rule</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Main/Stock/D/20/02/C, Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>[PURCHARN] CB Charnwod Smoked Cheese 1/2 Wheel Pkg</t>
+          <t>[PURAUSPECPEP] CB AUSTRALIAN PECORINO PEPPER WHEL PKG</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -3831,29 +4423,39 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/F/14/02</t>
+          <t>No Putaway Rule</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Main/Stock, Main/Stock/H/06/02</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>[PURDANISHBLUE] CB Danish Blue Cheese Whel Pkg</t>
+          <t>[PURAUSPEC] CB AUSTRALIAN PECORINO WHEL PKG</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Main/Stock/F/14/02, Main/Stock/H/06/02, Main/Stock/N/06/01</t>
+          <t>No Putaway Rule</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Main/Stock, Main/Stock/H/06/02</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>[PUREDAMDUTCH] CB Dutch Edam Cheese Red Bal Pkg</t>
+          <t>[PURCHARN] CB Charnwod Smoked Cheese 1/2 Wheel Pkg</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3861,29 +4463,39 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Main/Stock/H/06/02, Main/Stock/N/06/01</t>
+          <t>No Putaway Rule</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Main/Stock, Main/Stock/F/14/02</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>[PURESROM] CB ESROM DANISH CHEESE FULL WHEL PKG</t>
+          <t>[PURDANISHBLUE] CB Danish Blue Cheese Whel Pkg</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/H/06/02</t>
+          <t>No Putaway Rule</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Main/Stock/F/14/02, Main/Stock/H/06/02, Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>[PURGOUDA] CB Gouda Cheese Full Whel Pkg</t>
+          <t>[PUREDAMDUTCH] CB Dutch Edam Cheese Red Bal Pkg</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3891,20 +4503,30 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Main/Stock/F/14/02, Main/Stock/H/06/02</t>
+          <t>No Putaway Rule</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Main/Stock/H/06/02, Main/Stock/N/06/01</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>[PURMANCHEGO12] CB MANCHEGO AGED 12 MONTHS WHEL PKG</t>
+          <t>[PURESROM] CB ESROM DANISH CHEESE FULL WHEL PKG</t>
         </is>
       </c>
       <c r="B62" t="n">
         <v>2</v>
       </c>
       <c r="C62" t="inlineStr">
+        <is>
+          <t>No Putaway Rule</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
         <is>
           <t>Main/Stock, Main/Stock/H/06/02</t>
         </is>
@@ -3913,13 +4535,18 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>[PURPROVDOL] CB PROVOLONE DOLCE FUL RW</t>
+          <t>[PURGOUDA] CB Gouda Cheese Full Whel Pkg</t>
         </is>
       </c>
       <c r="B63" t="n">
         <v>2</v>
       </c>
       <c r="C63" t="inlineStr">
+        <is>
+          <t>No Putaway Rule</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
         <is>
           <t>Main/Stock/F/14/02, Main/Stock/H/06/02</t>
         </is>
@@ -3928,13 +4555,18 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>[PURVINTAGEB] ENGLISH Vintage Chedar Wheel Pkg</t>
+          <t>[PURMANCHEGO12] CB MANCHEGO AGED 12 MONTHS WHEL PKG</t>
         </is>
       </c>
       <c r="B64" t="n">
         <v>2</v>
       </c>
       <c r="C64" t="inlineStr">
+        <is>
+          <t>No Putaway Rule</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
         <is>
           <t>Main/Stock, Main/Stock/H/06/02</t>
         </is>
@@ -3943,7 +4575,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>[PURWALNUT] CB Walnut Chese Wheel Pkg</t>
+          <t>[PURPROVDOL] CB PROVOLONE DOLCE FUL RW</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3951,14 +4583,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Main/Stock, Main/Stock/H/06/02</t>
+          <t>Main/Stock/H/06/01</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Main/Stock/F/14/02, Main/Stock/H/06/02</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>[SPGOATB] CB Spanish Goat Cheese Semihard Wheel Pkg</t>
+          <t>[PURVINTAGEB] ENGLISH Vintage Chedar Wheel Pkg</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -3966,20 +4603,70 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Main/Stock/F/14/02, Main/Stock/H/06/02</t>
+          <t>No Putaway Rule</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Main/Stock, Main/Stock/H/06/02</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
+          <t>[PURWALNUT] CB Walnut Chese Wheel Pkg</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>2</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>No Putaway Rule</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Main/Stock, Main/Stock/H/06/02</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>[SPGOATB] CB Spanish Goat Cheese Semihard Wheel Pkg</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>2</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Main/Stock/H/06/01</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Main/Stock/F/14/02, Main/Stock/H/06/02</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
           <t>[WALNUTB] CB Walnut Cheese Wheel Pkg</t>
         </is>
       </c>
-      <c r="B67" t="n">
-        <v>2</v>
-      </c>
-      <c r="C67" t="inlineStr">
+      <c r="B69" t="n">
+        <v>2</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Main/Stock/H/06/02</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
         <is>
           <t>Main/Stock/F/14/02, Main/Stock/H/06/02</t>
         </is>

</xml_diff>